<commit_message>
Migrate DE home page (/de)
- Import template `home` for https://www.amag.ch/de.html, reusing the en home
  blocks and variants (hero-carousel, quick-links, vehicle-search, news-cards
  grid + carousels, icon-feature-grid, newsletter-band, testimonial,
  pledge-row plain-head, accordion-faq)
- New blocks for the German-only sections: news-cards-articles (dated news
  list) and video-brand-film (Vimeo brand film, loads on play)
- New parsers; news-cards parser extended with carousel mode; cleanup and
  section transformers gated on the template so the garage import is unchanged
- metadata.json / README.md for hero-carousel, quick-links, newsletter-band,
  accordion-faq
- Header block synced with main (hover mega-menu, transparent home header)

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-garagenuebersicht.report.xlsx
+++ b/tools/importer/reports/import-garagenuebersicht.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,30 @@
     <t>url</t>
   </si>
   <si>
+    <t>de.report.json</t>
+  </si>
+  <si>
+    <t>["hero-carousel","quick-links","vehicle-search","news-cards","news-cards","news-cards","icon-feature-grid","news-cards-articles","newsletter-band","newsletter-band","video-brand-film","testimonial","pledge-row","accordion-faq"]</t>
+  </si>
+  <si>
+    <t>de</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>home</t>
+  </si>
+  <si>
+    <t>2026-10-19T18:52:54.342Z</t>
+  </si>
+  <si>
+    <t>Das grösste Automobilunternehmen der Schweiz | AMAG</t>
+  </si>
+  <si>
+    <t>https://www.amag.ch/de.html</t>
+  </si>
+  <si>
     <t>de/garagenuebersicht/garage-buelach.report.json</t>
   </si>
   <si>
@@ -46,13 +70,10 @@
     <t>de/garagenuebersicht/garage-buelach</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>garagenuebersicht</t>
   </si>
   <si>
-    <t>2026-10-14T14:03:42.740Z</t>
+    <t>2026-10-19T18:54:50.583Z</t>
   </si>
   <si>
     <t>🚗 Autohändler und Garage Bülach | AMAG</t>
@@ -447,7 +468,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="49" customWidth="1"/>
@@ -455,8 +476,7 @@
     <col min="3" max="3" width="37" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="41" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +529,32 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>